<commit_message>
Hogar de Refugio: juntas del colector renombradas (tecnopor y sellador asfaltico; entre colector y cerco perimetrico), sello elastomerico reemplazado por sellador asfaltico; sin cambio de cantidades
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/METRADO_DRENAJE_MUJERES_VIOLENTADAS.xlsx
+++ b/entregables/METRADO_DRENAJE_MUJERES_VIOLENTADAS.xlsx
@@ -50,7 +50,7 @@
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'PLANILLA GENERAL DE METRADOS'!$A$1:$L$322</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">RESUMEN!$A$1:$D$75</definedName>
   </definedNames>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -923,13 +923,13 @@
     <t xml:space="preserve">01.04.04.06.01</t>
   </si>
   <si>
-    <t xml:space="preserve">JUNTA DE DILATACION E=1" CON TECNOPOR Y SELLADOR ELASTOMERICO</t>
+    <t xml:space="preserve">JUNTA DE DILATACION E=1" CON TECNOPOR Y SELLADOR ASFALTICO EN COLECTOR</t>
   </si>
   <si>
     <t xml:space="preserve">01.04.04.06.02</t>
   </si>
   <si>
-    <t xml:space="preserve">JUNTA E=1" CON TECNOPOR ENTRE COLECTOR Y PISO ADYACENTE</t>
+    <t xml:space="preserve">JUNTA E=1" CON TECNOPOR ENTRE COLECTOR Y CERCO PERIMETRICO</t>
   </si>
   <si>
     <t xml:space="preserve">ITEM</t>
@@ -3245,7 +3245,7 @@
     <t xml:space="preserve">COLECTOR PLUVIAL FRONTAL - JUNTAS Y EMPALMES DE CUNETAS</t>
   </si>
   <si>
-    <t xml:space="preserve">Lamina DP-01 (nota 5), DP-03 y DP-06C. Junta de dilatacion de 1" cada 4.00 m en todo el perimetro de la seccion (tecnopor + sellador elastomerico). Junta de tecnopor de 1" entre el colector y el cimiento del cerco, y entre el borde de la losa y el piso adyacente. Empalme de cada cuneta por ventana en el muro lado predio con caida libre al fondo (sin dintel adicional).</t>
+    <t xml:space="preserve">Lamina DP-01 (nota 5), DP-03 y DP-06C. Junta de dilatacion de 1" cada 4.00 m en todo el perimetro de la seccion (tecnopor de 1" en todo el perimetro + sellador asfaltico RC-250 con arena de 1" x 2" en la cara expuesta, EG-2013 secc. 510.02 c y 438.02 e 3). Junta de tecnopor de 1" entre el colector y el cimiento del cerco, y entre el borde de la losa y el piso adyacente. Empalme de cada cuneta por ventana en el muro lado predio con caida libre al fondo (sin dintel adicional).</t>
   </si>
   <si>
     <t xml:space="preserve">PROGRESIVA / DETALLE</t>
@@ -3254,7 +3254,7 @@
     <t xml:space="preserve">PARCIAL (m)</t>
   </si>
   <si>
-    <t xml:space="preserve">JUNTA DE DILATACION e=1" CON TECNOPOR Y SELLADOR ELASTOMERICO (perimetro = 2 x ancho exterior + 2 x (e fondo + h max + e losa))</t>
+    <t xml:space="preserve">JUNTA DE DILATACION e=1" CON TECNOPOR Y SELLADOR ASFALTICO EN COLECTOR (perimetro = 2 x ancho exterior + 2 x (e fondo + h max + e losa))</t>
   </si>
   <si>
     <t xml:space="preserve">Juntas de dilatacion cada 4.00 m entre 0+004.00 y 0+068.00</t>
@@ -3266,7 +3266,7 @@
     <t xml:space="preserve">TOTAL JUNTA DE DILATACION (m)</t>
   </si>
   <si>
-    <t xml:space="preserve">JUNTA DE TECNOPOR e=1" ENTRE COLECTOR, CERCO Y PISO ADYACENTE</t>
+    <t xml:space="preserve">JUNTA e=1" CON TECNOPOR ENTRE COLECTOR Y CERCO PERIMETRICO</t>
   </si>
   <si>
     <t xml:space="preserve">Contra el cimiento del cerco (tramo pegado al cerco, 0+000 a primer quiebre)</t>
@@ -3479,16 +3479,16 @@
     <t xml:space="preserve">glb</t>
   </si>
   <si>
-    <t xml:space="preserve">01.04.04.06.01 JUNTA DE DILATACION e=1" CON SELLADOR</t>
+    <t xml:space="preserve">01.04.04.06.01 JUNTA DE DILATACION e=1" CON TECNOPOR Y SELLADOR ASFALTICO</t>
   </si>
   <si>
     <t xml:space="preserve">Tecnopor 1"</t>
   </si>
   <si>
-    <t xml:space="preserve">Sello elastomerico de poliuretano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">01.04.04.06.02 JUNTA DE TECNOPOR e=1"</t>
+    <t xml:space="preserve">Sellador asfaltico: asfalto liquido RC-250 + arena gruesa (sello de 1" x 2")</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01.04.04.06.02 JUNTA e=1" CON TECNOPOR ENTRE COLECTOR Y CERCO PERIMETRICO</t>
   </si>
   <si>
     <t xml:space="preserve">ANALISIS DE COSTO UNITARIO - TAPA DE REGISTRO 0.68 x 0.68 C/MARCO Y CONTRAMARCO</t>
@@ -26828,15 +26828,17 @@
       <c r="E69" s="295" t="s">
         <v>987</v>
       </c>
-      <c r="F69" s="285" t="s">
-        <v>50</v>
+      <c r="F69" s="285" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
       </c>
       <c r="G69" s="284" t="n">
-        <v>0.35</v>
+        <v>0.0013</v>
       </c>
       <c r="H69" s="296" t="n">
         <f aca="false">G69*$D$68</f>
-        <v>35.224</v>
+        <v>0.130832</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Hogar de Refugio: hojas ACU JUNTA DILATACION y ACU JUNTA CERCO dentro de la planilla
Cantidades por metro tomadas de la lamina DD-03 (tecnopor 1" y sellador asfaltico 1" x 2" de RC-250
+ arena) y de la hoja COLECTOR JUNTAS Y EMPALMES; precios con su fuente (tecnopor Sodimac, RC-250
Conselva). COLECTOR INSUMOS lee de las ACU el tecnopor y la mezcla del sellador. Metrados sin cambio.
Se retira la ACU aparte de la junta con el cerco (reemplazada por la hoja de la planilla).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/METRADO_DRENAJE_MUJERES_VIOLENTADAS.xlsx
+++ b/entregables/METRADO_DRENAJE_MUJERES_VIOLENTADAS.xlsx
@@ -34,6 +34,8 @@
     <sheet name="ACU TAPA REGISTRO" sheetId="24" state="visible" r:id="rId26"/>
     <sheet name="ACU CANALETAS" sheetId="25" state="visible" r:id="rId27"/>
     <sheet name="DESAGREGADO TAPA REGISTRO" sheetId="26" state="visible" r:id="rId28"/>
+    <sheet name="ACU JUNTA DILATACION" sheetId="27" state="visible" r:id="rId30"/>
+    <sheet name="ACU JUNTA CERCO" sheetId="28" state="visible" r:id="rId31"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="24" name="_xlnm.Print_Area" vbProcedure="false">'ACU CANALETAS'!$A$1:$H$111</definedName>
@@ -510,7 +512,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3401" uniqueCount="1222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3401" uniqueCount="1294">
   <si>
     <t xml:space="preserve">RESUMEN METRADOS DE DRENAJE PLUVIAL</t>
   </si>
@@ -4188,6 +4190,222 @@
   </si>
   <si>
     <t xml:space="preserve">Analisis de la partida de Delphin 01.04.04.06.05.01 TAPA DE REGISTRO 0.68x0.68 C/MARCO Y CONTRAMARCO, partida 01.04.04.05.01 del metrado; componentes desagregados en la hoja DESAGREGADO TAPA REGISTRO. Cantidad por tapa = metrado del componente / numero de tapas. Ratios de insumos tomados de la hoja COLECTOR INSUMOS. Celda amarilla = dato (ratio o precio); verde = formula. Precios sin IGV obtenidos de precios publicados (octubre 2026), con su fuente en la columna H; los marcados "por cotizar" deben confirmarse en Tarapoto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANALISIS DE COSTO UNITARIO - JUNTA DE DILATACION E=1" CON TECNOPOR Y SELLADOR ASFALTICO EN COLECTOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partida de Delphin 01.04.04.06.01 JUNTA DE DILATACION E=1" CON TECNOPOR Y SELLADOR ASFALTICO EN COLECTOR (metrado 01.04.04.06.01, hoja COLECTOR JUNTAS Y EMPALMES). Se mide por metro de junta a lo largo del perimetro de la seccion. Cantidades de la lamina DD-03: plancha de tecnopor de 1" en toda la seccion y sellador asfaltico 1" x 2" (asfalto liquido RC-250 + arena gruesa) en las caras interiores y en la cara superior (EG-2013 MTC, 510). Celda amarilla = dato; verde = formula. Precios sin IGV.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. CANTIDADES POR METRO DE JUNTA (lamina DD-03 y hoja COLECTOR JUNTAS Y EMPALMES)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONCEPTO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perimetro de la seccion en cada junta: 2 x 1.10 + 2 x (0.15 + 1.61 + 0.10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COLECTOR JUNTAS Y EMPALMES fila 11; DD-03 A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Numero de juntas de dilatacion (cada 4.00 m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COLECTOR JUNTAS Y EMPALMES fila 11; DD-03 E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Area de tecnopor por junta: seccion 1.10 x 1.86 menos el hueco 0.80 x 1.61</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DD-03, cuadro de componentes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tecnopor por metro de junta (area neta)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">formula</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desperdicio por el corte del anillo en planchas de 1.20 x 2.40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">criterio: recortes del hueco interior y de las esquinas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Area de una plancha de tecnopor 1" (1.20 x 2.40 m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">medida comercial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planchas de tecnopor por metro de junta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pln/m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Longitud sellada por junta: caras interiores 2 x 1.61 + 0.80 y cara superior 1.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seccion del sellador 1" x 2" (0.0254 x 0.0508)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DD-03 B; EG-2013 510.02 c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mezcla de sellador por metro de junta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m3/m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asfalto liquido RC-250 por m3 de mezcla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gal/m3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">criterio: mezcla de ~2,000 kg/m3 con ~9 % de asfalto = 180 kg / 3.6 kg/gal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arena gruesa por m3 de mezcla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m3/m3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">criterio: arena suelta con 5 % de desperdicio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operario por metro de junta (colocacion del tecnopor y sellado)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hh/m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COLECTOR INSUMOS fila 71</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peon por metro de junta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COLECTOR INSUMOS fila 72</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. ANALISIS DE COSTO UNITARIO (formato Delphin)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01.04.04.06.01 JUNTA DE DILATACION E=1" CON TECNOPOR Y SELLADOR ASFALTICO EN COLECTOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01.04.04.06.01 (hoja COLECTOR JUNTAS Y EMPALMES)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rendimiento (m/dia, cuadrilla de 1 operario)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CANTIDAD POR M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">costo hora-hombre de la ACU TAPA REGISTRO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plancha de tecnopor 1" x 1.20 x 2.40 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pln</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sodimac Peru: plancha de poliestireno expandido 1" x 1.20 x 2.40 m (Dipropor) S/ 13.90 con IGV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asfalto liquido RC-250</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conselva: asfalto liquido RC-250 por galon S/ 17.70 con IGV (Petroperu publica su lista ex planta; confirmar en Tarapoto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">precio de la ACU TAPA REGISTRO (Agregados Tarapoto, Morales)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 % del costo de mano de obra (incluye recipiente para calentar el asfalto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COSTO DIRECTO DE LA PARTIDA (metrado x costo unitario, S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANALISIS DE COSTO UNITARIO - JUNTA E=1" CON TECNOPOR Y SELLADOR ASFALTICO ENTRE COLECTOR Y CERCO PERIMETRICO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partida de Delphin 01.04.04.06.02 JUNTA E=1" CON TECNOPOR Y SELLADOR ASFALTICO ENTRE COLECTOR Y CERCO PERIMETRICO (metrado 01.04.04.06.02, hoja COLECTOR JUNTAS Y EMPALMES). Cantidades de la lamina DD-03: plancha de tecnopor de 1" de 0.90 m de altura contra el cimiento del cerco y de 0.10 m en el borde de la losa con el piso adyacente, con sellador asfaltico 1" x 2" (RC-250 + arena) en la cara superior. Celda amarilla = dato; verde = formula. Precios sin IGV.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Junta contra el cimiento del cerco (0+000.00 a 0+058.81)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COLECTOR JUNTAS Y EMPALMES fila 15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Altura de la plancha contra el cerco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DD-03 C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Junta en el borde de la losa con el piso adyacente (colector y cajas CL y CC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COLECTOR JUNTAS Y EMPALMES filas 16 a 18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Altura de la plancha en el borde de la losa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DD-03 D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Longitud total de la partida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COLECTOR JUNTAS Y EMPALMES fila 19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tecnopor por metro de junta (promedio ponderado)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desperdicio por el corte en tiras</t>
+  </si>
+  <si>
+    <t xml:space="preserve">criterio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mezcla de sellador por metro de junta: 1" x 2" en la cara superior (0.0254 x 0.0508)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DD-03 C y D; EG-2013 510.02 c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peon por metro de junta (corte y colocacion de las tiras)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COLECTOR INSUMOS fila 74</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operario por metro de junta (sellado)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COLECTOR INSUMOS fila 76</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01.04.04.06.02 JUNTA E=1" CON TECNOPOR Y SELLADOR ASFALTICO ENTRE COLECTOR Y CERCO PERIMETRICO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01.04.04.06.02 (hoja COLECTOR JUNTAS Y EMPALMES)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rendimiento (m/dia, operario de sellado)</t>
   </si>
 </sst>
 </file>
@@ -4981,7 +5199,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="309">
+  <cellXfs count="310">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -6218,6 +6436,10 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="170" fontId="24" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -26945,12 +27167,13 @@
       <c r="F69" s="285" t="s">
         <v>168</v>
       </c>
-      <c r="G69" s="284" t="n">
-        <v>0.25</v>
+      <c r="G69" s="306" t="n">
+        <f aca="false">'ACU JUNTA DILATACION'!$D$14*(1+'ACU JUNTA DILATACION'!$D$15)</f>
+        <v>0.140844594594595</v>
       </c>
       <c r="H69" s="296" t="n">
         <f aca="false">G69*$D$69</f>
-        <v>25.16</v>
+        <v>14.1746</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26966,12 +27189,13 @@
           <t>m3</t>
         </is>
       </c>
-      <c r="G70" s="284" t="n">
-        <v>0.0013</v>
+      <c r="G70" s="306" t="n">
+        <f aca="false">'ACU JUNTA DILATACION'!$D$20</f>
+        <v>0.00111595243243243</v>
       </c>
       <c r="H70" s="296" t="n">
         <f aca="false">G70*$D$69</f>
-        <v>0.130832</v>
+        <v>0.1123094528</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27032,12 +27256,13 @@
       <c r="F73" s="285" t="s">
         <v>168</v>
       </c>
-      <c r="G73" s="284" t="n">
-        <v>0.15</v>
+      <c r="G73" s="306" t="n">
+        <f aca="false">'ACU JUNTA CERCO'!$D$16*(1+'ACU JUNTA CERCO'!$D$17)</f>
+        <v>0.339128515160277</v>
       </c>
       <c r="H73" s="296" t="n">
         <f aca="false">G73*$D$73</f>
-        <v>31.64685</v>
+        <v>71.548995</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27072,12 +27297,13 @@
           <t>m3</t>
         </is>
       </c>
-      <c r="G75" s="284" t="n">
-        <v>0.0013</v>
+      <c r="G75" s="306" t="n">
+        <f aca="false">'ACU JUNTA CERCO'!$D$20</f>
+        <v>0.00129032</v>
       </c>
       <c r="H75" s="296" t="n">
         <f aca="false">G75*$D$73</f>
-        <v>0.2742727</v>
+        <v>0.27223042328</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -32149,6 +32375,1702 @@
     <mergeCell ref="B31:G31"/>
     <mergeCell ref="B37:G37"/>
     <mergeCell ref="A41:G41"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:H46"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="44"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="277" t="s">
+        <v>1222</v>
+      </c>
+      <c r="B1" s="277"/>
+      <c r="C1" s="277"/>
+      <c r="D1" s="277"/>
+      <c r="E1" s="277"/>
+      <c r="F1" s="277"/>
+      <c r="G1" s="277"/>
+      <c r="H1" s="277"/>
+    </row>
+    <row r="2" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="278" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="278"/>
+      <c r="C2" s="279" t="str">
+        <f aca="false">+RESUMEN!B4</f>
+        <v>GERENCIA TERRITORIAL BAJO MAYO - TARAPOTO</v>
+      </c>
+      <c r="D2" s="279"/>
+      <c r="E2" s="279"/>
+      <c r="F2" s="279"/>
+      <c r="G2" s="279"/>
+      <c r="H2" s="279"/>
+    </row>
+    <row r="3" customFormat="false" ht="58.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="278" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="278"/>
+      <c r="C3" s="279" t="str">
+        <f aca="false">+RESUMEN!B5</f>
+        <v>“CREACIÓN DEL SERVICIO DE PROTECCIÓN A MUJERES VÍCTIMAS DE VIOLENCIA EN SITUACIÓN DE RIESGO DE FEMINICIDIO O PELIGRE SU INTEGRIDAD Y/O SALUD FÍSICA Y/O MENTAL EN HOGAR DE REFUGIO TEMPORAL DISTRITO DE MORALES DE LA PROVINCIA DE SAN MARTÍN DEL DEPARTAMENTO DE SAN MARTÍN”, con CUI N.° 2675514</v>
+      </c>
+      <c r="D3" s="279"/>
+      <c r="E3" s="279"/>
+      <c r="F3" s="279"/>
+      <c r="G3" s="279"/>
+      <c r="H3" s="279"/>
+    </row>
+    <row r="4" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="278" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="278"/>
+      <c r="C4" s="279" t="str">
+        <f aca="false">+RESUMEN!B6</f>
+        <v>SAN MARTIN - SAN MARTIN - MORALES</v>
+      </c>
+      <c r="D4" s="279"/>
+      <c r="E4" s="279"/>
+      <c r="F4" s="279"/>
+      <c r="G4" s="279"/>
+      <c r="H4" s="279"/>
+    </row>
+    <row r="5" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="278" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="278"/>
+      <c r="C5" s="280" t="n">
+        <f aca="false">+RESUMEN!B7</f>
+        <v>46266</v>
+      </c>
+      <c r="D5" s="280"/>
+      <c r="E5" s="280"/>
+      <c r="F5" s="280"/>
+      <c r="G5" s="280"/>
+      <c r="H5" s="280"/>
+    </row>
+    <row r="7" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="281" t="s">
+        <v>1223</v>
+      </c>
+      <c r="B7" s="281"/>
+      <c r="C7" s="281"/>
+      <c r="D7" s="281"/>
+      <c r="E7" s="281"/>
+      <c r="F7" s="281"/>
+      <c r="G7" s="281"/>
+      <c r="H7" s="281"/>
+    </row>
+    <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="294" t="s">
+        <v>1224</v>
+      </c>
+      <c r="B9" s="294"/>
+      <c r="C9" s="294"/>
+      <c r="D9" s="294"/>
+      <c r="E9" s="294"/>
+      <c r="F9" s="294"/>
+      <c r="G9" s="294"/>
+      <c r="H9" s="294"/>
+    </row>
+    <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="282" t="s">
+        <v>331</v>
+      </c>
+      <c r="B10" s="282" t="s">
+        <v>1225</v>
+      </c>
+      <c r="C10" s="282" t="s">
+        <v>151</v>
+      </c>
+      <c r="D10" s="282" t="s">
+        <v>292</v>
+      </c>
+      <c r="E10" s="282"/>
+      <c r="F10" s="282"/>
+      <c r="G10" s="282"/>
+      <c r="H10" s="282" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="283" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="B11" s="149" t="s">
+        <v>1226</v>
+      </c>
+      <c r="C11" s="285" t="s">
+        <v>57</v>
+      </c>
+      <c r="D11" s="306" t="n">
+        <f aca="false">'COLECTOR JUNTAS Y EMPALMES'!E11</f>
+        <v>5.92</v>
+      </c>
+      <c r="E11" s="295"/>
+      <c r="F11" s="295"/>
+      <c r="G11" s="295"/>
+      <c r="H11" s="149" t="s">
+        <v>1227</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="283" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="B12" s="149" t="s">
+        <v>1228</v>
+      </c>
+      <c r="C12" s="285" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" s="306" t="n">
+        <f aca="false">'COLECTOR JUNTAS Y EMPALMES'!D11</f>
+        <v>17.0</v>
+      </c>
+      <c r="E12" s="295"/>
+      <c r="F12" s="295"/>
+      <c r="G12" s="295"/>
+      <c r="H12" s="149" t="s">
+        <v>1229</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="283" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="B13" s="149" t="s">
+        <v>1230</v>
+      </c>
+      <c r="C13" s="285" t="s">
+        <v>168</v>
+      </c>
+      <c r="D13" s="306" t="n">
+        <f aca="false">1.10*(0.15+1.61+0.10)-0.80*1.61</f>
+        <v>0.758</v>
+      </c>
+      <c r="E13" s="295"/>
+      <c r="F13" s="295"/>
+      <c r="G13" s="295"/>
+      <c r="H13" s="149" t="s">
+        <v>1231</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="283" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="B14" s="149" t="s">
+        <v>1232</v>
+      </c>
+      <c r="C14" s="285" t="s">
+        <v>602</v>
+      </c>
+      <c r="D14" s="306" t="n">
+        <f aca="false">D13/D11</f>
+        <v>0.128040540540541</v>
+      </c>
+      <c r="E14" s="295"/>
+      <c r="F14" s="295"/>
+      <c r="G14" s="295"/>
+      <c r="H14" s="149" t="s">
+        <v>1233</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="283" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="B15" s="149" t="s">
+        <v>1234</v>
+      </c>
+      <c r="C15" s="285" t="s">
+        <v>523</v>
+      </c>
+      <c r="D15" s="309" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E15" s="295"/>
+      <c r="F15" s="295"/>
+      <c r="G15" s="295"/>
+      <c r="H15" s="149" t="s">
+        <v>1235</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="283" t="n">
+        <v>6.0</v>
+      </c>
+      <c r="B16" s="149" t="s">
+        <v>1236</v>
+      </c>
+      <c r="C16" s="285" t="s">
+        <v>168</v>
+      </c>
+      <c r="D16" s="309" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="E16" s="295"/>
+      <c r="F16" s="295"/>
+      <c r="G16" s="295"/>
+      <c r="H16" s="149" t="s">
+        <v>1237</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="283" t="n">
+        <v>7.0</v>
+      </c>
+      <c r="B17" s="149" t="s">
+        <v>1238</v>
+      </c>
+      <c r="C17" s="285" t="s">
+        <v>1239</v>
+      </c>
+      <c r="D17" s="306" t="n">
+        <f aca="false">D14*(1+D15)/D16</f>
+        <v>0.0489043731231231</v>
+      </c>
+      <c r="E17" s="295"/>
+      <c r="F17" s="295"/>
+      <c r="G17" s="295"/>
+      <c r="H17" s="149" t="s">
+        <v>1233</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="283" t="n">
+        <v>8.0</v>
+      </c>
+      <c r="B18" s="149" t="s">
+        <v>1240</v>
+      </c>
+      <c r="C18" s="285" t="s">
+        <v>57</v>
+      </c>
+      <c r="D18" s="306" t="n">
+        <f aca="false">2*1.61+0.80+1.10</f>
+        <v>5.12</v>
+      </c>
+      <c r="E18" s="295"/>
+      <c r="F18" s="295"/>
+      <c r="G18" s="295"/>
+      <c r="H18" s="149" t="s">
+        <v>1231</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="283" t="n">
+        <v>9.0</v>
+      </c>
+      <c r="B19" s="149" t="s">
+        <v>1241</v>
+      </c>
+      <c r="C19" s="285" t="s">
+        <v>168</v>
+      </c>
+      <c r="D19" s="306" t="n">
+        <f aca="false">0.0254*0.0508</f>
+        <v>0.00129032</v>
+      </c>
+      <c r="E19" s="295"/>
+      <c r="F19" s="295"/>
+      <c r="G19" s="295"/>
+      <c r="H19" s="149" t="s">
+        <v>1242</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="283" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="B20" s="149" t="s">
+        <v>1243</v>
+      </c>
+      <c r="C20" s="285" t="s">
+        <v>1244</v>
+      </c>
+      <c r="D20" s="306" t="n">
+        <f aca="false">D19*D18/D11</f>
+        <v>0.00111595243243243</v>
+      </c>
+      <c r="E20" s="295"/>
+      <c r="F20" s="295"/>
+      <c r="G20" s="295"/>
+      <c r="H20" s="149" t="s">
+        <v>1233</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="283" t="n">
+        <v>11.0</v>
+      </c>
+      <c r="B21" s="149" t="s">
+        <v>1245</v>
+      </c>
+      <c r="C21" s="285" t="s">
+        <v>1246</v>
+      </c>
+      <c r="D21" s="309" t="n">
+        <v>50.0</v>
+      </c>
+      <c r="E21" s="295"/>
+      <c r="F21" s="295"/>
+      <c r="G21" s="295"/>
+      <c r="H21" s="149" t="s">
+        <v>1247</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="283" t="n">
+        <v>12.0</v>
+      </c>
+      <c r="B22" s="149" t="s">
+        <v>1248</v>
+      </c>
+      <c r="C22" s="285" t="s">
+        <v>1249</v>
+      </c>
+      <c r="D22" s="309" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E22" s="295"/>
+      <c r="F22" s="295"/>
+      <c r="G22" s="295"/>
+      <c r="H22" s="149" t="s">
+        <v>1250</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="283" t="n">
+        <v>13.0</v>
+      </c>
+      <c r="B23" s="149" t="s">
+        <v>1251</v>
+      </c>
+      <c r="C23" s="285" t="s">
+        <v>1252</v>
+      </c>
+      <c r="D23" s="306" t="n">
+        <f aca="false">'COLECTOR INSUMOS'!G71</f>
+        <v>0.2</v>
+      </c>
+      <c r="E23" s="295"/>
+      <c r="F23" s="295"/>
+      <c r="G23" s="295"/>
+      <c r="H23" s="149" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="283" t="n">
+        <v>14.0</v>
+      </c>
+      <c r="B24" s="149" t="s">
+        <v>1254</v>
+      </c>
+      <c r="C24" s="285" t="s">
+        <v>1252</v>
+      </c>
+      <c r="D24" s="306" t="n">
+        <f aca="false">'COLECTOR INSUMOS'!G72</f>
+        <v>0.2</v>
+      </c>
+      <c r="E24" s="295"/>
+      <c r="F24" s="295"/>
+      <c r="G24" s="295"/>
+      <c r="H24" s="149" t="s">
+        <v>1255</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="294" t="s">
+        <v>1256</v>
+      </c>
+      <c r="B26" s="294"/>
+      <c r="C26" s="294"/>
+      <c r="D26" s="294"/>
+      <c r="E26" s="294"/>
+      <c r="F26" s="294"/>
+      <c r="G26" s="294"/>
+      <c r="H26" s="294"/>
+    </row>
+    <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="294" t="s">
+        <v>1056</v>
+      </c>
+      <c r="B27" s="294"/>
+      <c r="C27" s="295" t="s">
+        <v>1257</v>
+      </c>
+      <c r="D27" s="295"/>
+      <c r="E27" s="295"/>
+      <c r="F27" s="295"/>
+      <c r="G27" s="295"/>
+      <c r="H27" s="295"/>
+    </row>
+    <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="294" t="s">
+        <v>1058</v>
+      </c>
+      <c r="B28" s="294"/>
+      <c r="C28" s="295" t="s">
+        <v>1258</v>
+      </c>
+      <c r="D28" s="295"/>
+      <c r="E28" s="295"/>
+      <c r="F28" s="295"/>
+      <c r="G28" s="295"/>
+      <c r="H28" s="295"/>
+    </row>
+    <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="294" t="s">
+        <v>502</v>
+      </c>
+      <c r="B29" s="294"/>
+      <c r="C29" s="295" t="s">
+        <v>57</v>
+      </c>
+      <c r="D29" s="295"/>
+      <c r="E29" s="295"/>
+      <c r="F29" s="295"/>
+      <c r="G29" s="295"/>
+      <c r="H29" s="295"/>
+    </row>
+    <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="294" t="s">
+        <v>1060</v>
+      </c>
+      <c r="B30" s="294"/>
+      <c r="C30" s="290" t="n">
+        <f aca="false">'COLECTOR JUNTAS Y EMPALMES'!F12</f>
+        <v>100.64</v>
+      </c>
+      <c r="D30" s="290"/>
+      <c r="E30" s="290"/>
+      <c r="F30" s="290"/>
+      <c r="G30" s="290"/>
+      <c r="H30" s="290"/>
+    </row>
+    <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="294" t="s">
+        <v>1259</v>
+      </c>
+      <c r="B31" s="294"/>
+      <c r="C31" s="290" t="n">
+        <f aca="false">8/E34</f>
+        <v>40.0</v>
+      </c>
+      <c r="D31" s="290"/>
+      <c r="E31" s="290"/>
+      <c r="F31" s="290"/>
+      <c r="G31" s="290"/>
+      <c r="H31" s="290"/>
+    </row>
+    <row r="32" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="282" t="s">
+        <v>331</v>
+      </c>
+      <c r="B32" s="282" t="s">
+        <v>1062</v>
+      </c>
+      <c r="C32" s="282" t="s">
+        <v>151</v>
+      </c>
+      <c r="D32" s="282" t="s">
+        <v>1063</v>
+      </c>
+      <c r="E32" s="282" t="s">
+        <v>1260</v>
+      </c>
+      <c r="F32" s="282" t="s">
+        <v>1064</v>
+      </c>
+      <c r="G32" s="282" t="s">
+        <v>1020</v>
+      </c>
+      <c r="H32" s="282" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="21"/>
+      <c r="B33" s="294" t="s">
+        <v>1066</v>
+      </c>
+      <c r="C33" s="294"/>
+      <c r="D33" s="294"/>
+      <c r="E33" s="294"/>
+      <c r="F33" s="294"/>
+      <c r="G33" s="294"/>
+      <c r="H33" s="294"/>
+    </row>
+    <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="283" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="B34" s="295" t="s">
+        <v>952</v>
+      </c>
+      <c r="C34" s="285" t="s">
+        <v>953</v>
+      </c>
+      <c r="D34" s="306" t="n">
+        <f aca="false">E34*$C$31/8</f>
+        <v>1.0</v>
+      </c>
+      <c r="E34" s="306" t="n">
+        <f aca="false">$D$23</f>
+        <v>0.2</v>
+      </c>
+      <c r="F34" s="290" t="n">
+        <f aca="false">'ACU TAPA REGISTRO'!F69</f>
+        <v>30.42</v>
+      </c>
+      <c r="G34" s="290" t="n">
+        <f aca="false">E34*F34</f>
+        <v>6.084</v>
+      </c>
+      <c r="H34" s="149" t="s">
+        <v>1261</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="283" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="B35" s="295" t="s">
+        <v>955</v>
+      </c>
+      <c r="C35" s="285" t="s">
+        <v>953</v>
+      </c>
+      <c r="D35" s="306" t="n">
+        <f aca="false">E35*$C$31/8</f>
+        <v>1.0</v>
+      </c>
+      <c r="E35" s="306" t="n">
+        <f aca="false">$D$24</f>
+        <v>0.2</v>
+      </c>
+      <c r="F35" s="290" t="n">
+        <f aca="false">'ACU TAPA REGISTRO'!F71</f>
+        <v>20.79</v>
+      </c>
+      <c r="G35" s="290" t="n">
+        <f aca="false">E35*F35</f>
+        <v>4.158</v>
+      </c>
+      <c r="H35" s="149" t="s">
+        <v>1261</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="21"/>
+      <c r="B36" s="294" t="s">
+        <v>1068</v>
+      </c>
+      <c r="C36" s="295"/>
+      <c r="D36" s="295"/>
+      <c r="E36" s="295"/>
+      <c r="F36" s="295"/>
+      <c r="G36" s="296" t="n">
+        <f aca="false">SUM(G34:G35)</f>
+        <v>10.242</v>
+      </c>
+      <c r="H36" s="295"/>
+    </row>
+    <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="21"/>
+      <c r="B37" s="294" t="s">
+        <v>1069</v>
+      </c>
+      <c r="C37" s="294"/>
+      <c r="D37" s="294"/>
+      <c r="E37" s="294"/>
+      <c r="F37" s="294"/>
+      <c r="G37" s="294"/>
+      <c r="H37" s="294"/>
+    </row>
+    <row r="38" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="283" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="B38" s="295" t="s">
+        <v>1262</v>
+      </c>
+      <c r="C38" s="285" t="s">
+        <v>1263</v>
+      </c>
+      <c r="D38" s="295"/>
+      <c r="E38" s="306" t="n">
+        <f aca="false">$D$17</f>
+        <v>0.0489043731231231</v>
+      </c>
+      <c r="F38" s="290" t="n">
+        <f aca="false">13.9/1.18</f>
+        <v>11.7796610169492</v>
+      </c>
+      <c r="G38" s="290" t="n">
+        <f aca="false">E38*F38</f>
+        <v>0.57607693763679</v>
+      </c>
+      <c r="H38" s="149" t="s">
+        <v>1264</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="283" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="B39" s="295" t="s">
+        <v>1265</v>
+      </c>
+      <c r="C39" s="285" t="s">
+        <v>981</v>
+      </c>
+      <c r="D39" s="295"/>
+      <c r="E39" s="306" t="n">
+        <f aca="false">$D$20*$D$21</f>
+        <v>0.0557976216216216</v>
+      </c>
+      <c r="F39" s="290" t="n">
+        <f aca="false">17.7/1.18</f>
+        <v>15.0</v>
+      </c>
+      <c r="G39" s="290" t="n">
+        <f aca="false">E39*F39</f>
+        <v>0.836964324324325</v>
+      </c>
+      <c r="H39" s="149" t="s">
+        <v>1266</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="283" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="B40" s="295" t="s">
+        <v>946</v>
+      </c>
+      <c r="C40" s="285" t="s">
+        <v>167</v>
+      </c>
+      <c r="D40" s="295"/>
+      <c r="E40" s="306" t="n">
+        <f aca="false">$D$20*$D$22</f>
+        <v>0.00117175005405405</v>
+      </c>
+      <c r="F40" s="290" t="n">
+        <f aca="false">'ACU TAPA REGISTRO'!F77</f>
+        <v>40.68</v>
+      </c>
+      <c r="G40" s="290" t="n">
+        <f aca="false">E40*F40</f>
+        <v>0.0476667921989189</v>
+      </c>
+      <c r="H40" s="149" t="s">
+        <v>1267</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="21"/>
+      <c r="B41" s="294" t="s">
+        <v>1071</v>
+      </c>
+      <c r="C41" s="295"/>
+      <c r="D41" s="295"/>
+      <c r="E41" s="295"/>
+      <c r="F41" s="295"/>
+      <c r="G41" s="296" t="n">
+        <f aca="false">SUM(G38:G40)</f>
+        <v>1.46070805416003</v>
+      </c>
+      <c r="H41" s="295"/>
+    </row>
+    <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="21"/>
+      <c r="B42" s="294" t="s">
+        <v>1072</v>
+      </c>
+      <c r="C42" s="294"/>
+      <c r="D42" s="294"/>
+      <c r="E42" s="294"/>
+      <c r="F42" s="294"/>
+      <c r="G42" s="294"/>
+      <c r="H42" s="294"/>
+    </row>
+    <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="283" t="n">
+        <v>6.0</v>
+      </c>
+      <c r="B43" s="295" t="s">
+        <v>969</v>
+      </c>
+      <c r="C43" s="285" t="s">
+        <v>970</v>
+      </c>
+      <c r="D43" s="295"/>
+      <c r="E43" s="284" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F43" s="290" t="n">
+        <f aca="false">+G36</f>
+        <v>10.242</v>
+      </c>
+      <c r="G43" s="290" t="n">
+        <f aca="false">E43*F43</f>
+        <v>0.30726</v>
+      </c>
+      <c r="H43" s="149" t="s">
+        <v>1268</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="21"/>
+      <c r="B44" s="294" t="s">
+        <v>1075</v>
+      </c>
+      <c r="C44" s="295"/>
+      <c r="D44" s="295"/>
+      <c r="E44" s="295"/>
+      <c r="F44" s="295"/>
+      <c r="G44" s="296" t="n">
+        <f aca="false">SUM(G43:G43)</f>
+        <v>0.30726</v>
+      </c>
+      <c r="H44" s="295"/>
+    </row>
+    <row r="45" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="294" t="s">
+        <v>1119</v>
+      </c>
+      <c r="B45" s="294"/>
+      <c r="C45" s="294"/>
+      <c r="D45" s="294"/>
+      <c r="E45" s="294"/>
+      <c r="F45" s="294"/>
+      <c r="G45" s="296" t="n">
+        <f aca="false">+G36+G41+G44</f>
+        <v>12.00996805416</v>
+      </c>
+      <c r="H45" s="295"/>
+    </row>
+    <row r="46" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="294" t="s">
+        <v>1269</v>
+      </c>
+      <c r="B46" s="294"/>
+      <c r="C46" s="294"/>
+      <c r="D46" s="294"/>
+      <c r="E46" s="294"/>
+      <c r="F46" s="294"/>
+      <c r="G46" s="296" t="n">
+        <f aca="false">G45*C30</f>
+        <v>1208.68318497067</v>
+      </c>
+      <c r="H46" s="295"/>
+    </row>
+  </sheetData>
+  <mergeCells count="27">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:H2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:H3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:H4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:H5"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="C27:H27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="C28:H28"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="C29:H29"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="C30:H30"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="C31:H31"/>
+    <mergeCell ref="B33:H33"/>
+    <mergeCell ref="B37:H37"/>
+    <mergeCell ref="B42:H42"/>
+    <mergeCell ref="A45:F45"/>
+    <mergeCell ref="A46:F46"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:H46"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="44"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="277" t="s">
+        <v>1270</v>
+      </c>
+      <c r="B1" s="277"/>
+      <c r="C1" s="277"/>
+      <c r="D1" s="277"/>
+      <c r="E1" s="277"/>
+      <c r="F1" s="277"/>
+      <c r="G1" s="277"/>
+      <c r="H1" s="277"/>
+    </row>
+    <row r="2" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="278" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="278"/>
+      <c r="C2" s="279" t="str">
+        <f aca="false">+RESUMEN!B4</f>
+        <v>GERENCIA TERRITORIAL BAJO MAYO - TARAPOTO</v>
+      </c>
+      <c r="D2" s="279"/>
+      <c r="E2" s="279"/>
+      <c r="F2" s="279"/>
+      <c r="G2" s="279"/>
+      <c r="H2" s="279"/>
+    </row>
+    <row r="3" customFormat="false" ht="58.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="278" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="278"/>
+      <c r="C3" s="279" t="str">
+        <f aca="false">+RESUMEN!B5</f>
+        <v>“CREACIÓN DEL SERVICIO DE PROTECCIÓN A MUJERES VÍCTIMAS DE VIOLENCIA EN SITUACIÓN DE RIESGO DE FEMINICIDIO O PELIGRE SU INTEGRIDAD Y/O SALUD FÍSICA Y/O MENTAL EN HOGAR DE REFUGIO TEMPORAL DISTRITO DE MORALES DE LA PROVINCIA DE SAN MARTÍN DEL DEPARTAMENTO DE SAN MARTÍN”, con CUI N.° 2675514</v>
+      </c>
+      <c r="D3" s="279"/>
+      <c r="E3" s="279"/>
+      <c r="F3" s="279"/>
+      <c r="G3" s="279"/>
+      <c r="H3" s="279"/>
+    </row>
+    <row r="4" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="278" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="278"/>
+      <c r="C4" s="279" t="str">
+        <f aca="false">+RESUMEN!B6</f>
+        <v>SAN MARTIN - SAN MARTIN - MORALES</v>
+      </c>
+      <c r="D4" s="279"/>
+      <c r="E4" s="279"/>
+      <c r="F4" s="279"/>
+      <c r="G4" s="279"/>
+      <c r="H4" s="279"/>
+    </row>
+    <row r="5" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="278" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="278"/>
+      <c r="C5" s="280" t="n">
+        <f aca="false">+RESUMEN!B7</f>
+        <v>46266</v>
+      </c>
+      <c r="D5" s="280"/>
+      <c r="E5" s="280"/>
+      <c r="F5" s="280"/>
+      <c r="G5" s="280"/>
+      <c r="H5" s="280"/>
+    </row>
+    <row r="7" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="281" t="s">
+        <v>1271</v>
+      </c>
+      <c r="B7" s="281"/>
+      <c r="C7" s="281"/>
+      <c r="D7" s="281"/>
+      <c r="E7" s="281"/>
+      <c r="F7" s="281"/>
+      <c r="G7" s="281"/>
+      <c r="H7" s="281"/>
+    </row>
+    <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="294" t="s">
+        <v>1224</v>
+      </c>
+      <c r="B9" s="294"/>
+      <c r="C9" s="294"/>
+      <c r="D9" s="294"/>
+      <c r="E9" s="294"/>
+      <c r="F9" s="294"/>
+      <c r="G9" s="294"/>
+      <c r="H9" s="294"/>
+    </row>
+    <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="282" t="s">
+        <v>331</v>
+      </c>
+      <c r="B10" s="282" t="s">
+        <v>1225</v>
+      </c>
+      <c r="C10" s="282" t="s">
+        <v>151</v>
+      </c>
+      <c r="D10" s="282" t="s">
+        <v>292</v>
+      </c>
+      <c r="E10" s="282"/>
+      <c r="F10" s="282"/>
+      <c r="G10" s="282"/>
+      <c r="H10" s="282" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="283" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="B11" s="149" t="s">
+        <v>1272</v>
+      </c>
+      <c r="C11" s="285" t="s">
+        <v>57</v>
+      </c>
+      <c r="D11" s="306" t="n">
+        <f aca="false">'COLECTOR JUNTAS Y EMPALMES'!F15</f>
+        <v>58.805</v>
+      </c>
+      <c r="E11" s="295"/>
+      <c r="F11" s="295"/>
+      <c r="G11" s="295"/>
+      <c r="H11" s="149" t="s">
+        <v>1273</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="283" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="B12" s="149" t="s">
+        <v>1274</v>
+      </c>
+      <c r="C12" s="285" t="s">
+        <v>57</v>
+      </c>
+      <c r="D12" s="309" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E12" s="295"/>
+      <c r="F12" s="295"/>
+      <c r="G12" s="295"/>
+      <c r="H12" s="149" t="s">
+        <v>1275</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="283" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="B13" s="149" t="s">
+        <v>1276</v>
+      </c>
+      <c r="C13" s="285" t="s">
+        <v>57</v>
+      </c>
+      <c r="D13" s="306" t="n">
+        <f aca="false">'COLECTOR JUNTAS Y EMPALMES'!F16+'COLECTOR JUNTAS Y EMPALMES'!F17+'COLECTOR JUNTAS Y EMPALMES'!F18</f>
+        <v>152.174</v>
+      </c>
+      <c r="E13" s="295"/>
+      <c r="F13" s="295"/>
+      <c r="G13" s="295"/>
+      <c r="H13" s="149" t="s">
+        <v>1277</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="283" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="B14" s="149" t="s">
+        <v>1278</v>
+      </c>
+      <c r="C14" s="285" t="s">
+        <v>57</v>
+      </c>
+      <c r="D14" s="309" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E14" s="295"/>
+      <c r="F14" s="295"/>
+      <c r="G14" s="295"/>
+      <c r="H14" s="149" t="s">
+        <v>1279</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="283" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="B15" s="149" t="s">
+        <v>1280</v>
+      </c>
+      <c r="C15" s="285" t="s">
+        <v>57</v>
+      </c>
+      <c r="D15" s="306" t="n">
+        <f aca="false">'COLECTOR JUNTAS Y EMPALMES'!F19</f>
+        <v>210.979</v>
+      </c>
+      <c r="E15" s="295"/>
+      <c r="F15" s="295"/>
+      <c r="G15" s="295"/>
+      <c r="H15" s="149" t="s">
+        <v>1281</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="283" t="n">
+        <v>6.0</v>
+      </c>
+      <c r="B16" s="149" t="s">
+        <v>1282</v>
+      </c>
+      <c r="C16" s="285" t="s">
+        <v>602</v>
+      </c>
+      <c r="D16" s="306" t="n">
+        <f aca="false">(D11*D12+D13*D14)/D15</f>
+        <v>0.322979538247883</v>
+      </c>
+      <c r="E16" s="295"/>
+      <c r="F16" s="295"/>
+      <c r="G16" s="295"/>
+      <c r="H16" s="149" t="s">
+        <v>1233</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="283" t="n">
+        <v>7.0</v>
+      </c>
+      <c r="B17" s="149" t="s">
+        <v>1283</v>
+      </c>
+      <c r="C17" s="285" t="s">
+        <v>523</v>
+      </c>
+      <c r="D17" s="309" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E17" s="295"/>
+      <c r="F17" s="295"/>
+      <c r="G17" s="295"/>
+      <c r="H17" s="149" t="s">
+        <v>1284</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="283" t="n">
+        <v>8.0</v>
+      </c>
+      <c r="B18" s="149" t="s">
+        <v>1236</v>
+      </c>
+      <c r="C18" s="285" t="s">
+        <v>168</v>
+      </c>
+      <c r="D18" s="309" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="E18" s="295"/>
+      <c r="F18" s="295"/>
+      <c r="G18" s="295"/>
+      <c r="H18" s="149" t="s">
+        <v>1237</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="283" t="n">
+        <v>9.0</v>
+      </c>
+      <c r="B19" s="149" t="s">
+        <v>1238</v>
+      </c>
+      <c r="C19" s="285" t="s">
+        <v>1239</v>
+      </c>
+      <c r="D19" s="306" t="n">
+        <f aca="false">D16*(1+D17)/D18</f>
+        <v>0.117752956652874</v>
+      </c>
+      <c r="E19" s="295"/>
+      <c r="F19" s="295"/>
+      <c r="G19" s="295"/>
+      <c r="H19" s="149" t="s">
+        <v>1233</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="283" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="B20" s="149" t="s">
+        <v>1285</v>
+      </c>
+      <c r="C20" s="285" t="s">
+        <v>1244</v>
+      </c>
+      <c r="D20" s="306" t="n">
+        <f aca="false">0.0254*0.0508</f>
+        <v>0.00129032</v>
+      </c>
+      <c r="E20" s="295"/>
+      <c r="F20" s="295"/>
+      <c r="G20" s="295"/>
+      <c r="H20" s="149" t="s">
+        <v>1286</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="283" t="n">
+        <v>11.0</v>
+      </c>
+      <c r="B21" s="149" t="s">
+        <v>1245</v>
+      </c>
+      <c r="C21" s="285" t="s">
+        <v>1246</v>
+      </c>
+      <c r="D21" s="309" t="n">
+        <v>50.0</v>
+      </c>
+      <c r="E21" s="295"/>
+      <c r="F21" s="295"/>
+      <c r="G21" s="295"/>
+      <c r="H21" s="149" t="s">
+        <v>1247</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="283" t="n">
+        <v>12.0</v>
+      </c>
+      <c r="B22" s="149" t="s">
+        <v>1248</v>
+      </c>
+      <c r="C22" s="285" t="s">
+        <v>1249</v>
+      </c>
+      <c r="D22" s="309" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E22" s="295"/>
+      <c r="F22" s="295"/>
+      <c r="G22" s="295"/>
+      <c r="H22" s="149" t="s">
+        <v>1250</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="283" t="n">
+        <v>13.0</v>
+      </c>
+      <c r="B23" s="149" t="s">
+        <v>1287</v>
+      </c>
+      <c r="C23" s="285" t="s">
+        <v>1252</v>
+      </c>
+      <c r="D23" s="306" t="n">
+        <f aca="false">'COLECTOR INSUMOS'!G74</f>
+        <v>0.1</v>
+      </c>
+      <c r="E23" s="295"/>
+      <c r="F23" s="295"/>
+      <c r="G23" s="295"/>
+      <c r="H23" s="149" t="s">
+        <v>1288</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="283" t="n">
+        <v>14.0</v>
+      </c>
+      <c r="B24" s="149" t="s">
+        <v>1289</v>
+      </c>
+      <c r="C24" s="285" t="s">
+        <v>1252</v>
+      </c>
+      <c r="D24" s="306" t="n">
+        <f aca="false">'COLECTOR INSUMOS'!G76</f>
+        <v>0.05</v>
+      </c>
+      <c r="E24" s="295"/>
+      <c r="F24" s="295"/>
+      <c r="G24" s="295"/>
+      <c r="H24" s="149" t="s">
+        <v>1290</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="294" t="s">
+        <v>1256</v>
+      </c>
+      <c r="B26" s="294"/>
+      <c r="C26" s="294"/>
+      <c r="D26" s="294"/>
+      <c r="E26" s="294"/>
+      <c r="F26" s="294"/>
+      <c r="G26" s="294"/>
+      <c r="H26" s="294"/>
+    </row>
+    <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="294" t="s">
+        <v>1056</v>
+      </c>
+      <c r="B27" s="294"/>
+      <c r="C27" s="295" t="s">
+        <v>1291</v>
+      </c>
+      <c r="D27" s="295"/>
+      <c r="E27" s="295"/>
+      <c r="F27" s="295"/>
+      <c r="G27" s="295"/>
+      <c r="H27" s="295"/>
+    </row>
+    <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="294" t="s">
+        <v>1058</v>
+      </c>
+      <c r="B28" s="294"/>
+      <c r="C28" s="295" t="s">
+        <v>1292</v>
+      </c>
+      <c r="D28" s="295"/>
+      <c r="E28" s="295"/>
+      <c r="F28" s="295"/>
+      <c r="G28" s="295"/>
+      <c r="H28" s="295"/>
+    </row>
+    <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="294" t="s">
+        <v>502</v>
+      </c>
+      <c r="B29" s="294"/>
+      <c r="C29" s="295" t="s">
+        <v>57</v>
+      </c>
+      <c r="D29" s="295"/>
+      <c r="E29" s="295"/>
+      <c r="F29" s="295"/>
+      <c r="G29" s="295"/>
+      <c r="H29" s="295"/>
+    </row>
+    <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="294" t="s">
+        <v>1060</v>
+      </c>
+      <c r="B30" s="294"/>
+      <c r="C30" s="290" t="n">
+        <f aca="false">'COLECTOR JUNTAS Y EMPALMES'!F19</f>
+        <v>210.979</v>
+      </c>
+      <c r="D30" s="290"/>
+      <c r="E30" s="290"/>
+      <c r="F30" s="290"/>
+      <c r="G30" s="290"/>
+      <c r="H30" s="290"/>
+    </row>
+    <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="294" t="s">
+        <v>1293</v>
+      </c>
+      <c r="B31" s="294"/>
+      <c r="C31" s="290" t="n">
+        <f aca="false">8/E34</f>
+        <v>160.0</v>
+      </c>
+      <c r="D31" s="290"/>
+      <c r="E31" s="290"/>
+      <c r="F31" s="290"/>
+      <c r="G31" s="290"/>
+      <c r="H31" s="290"/>
+    </row>
+    <row r="32" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="282" t="s">
+        <v>331</v>
+      </c>
+      <c r="B32" s="282" t="s">
+        <v>1062</v>
+      </c>
+      <c r="C32" s="282" t="s">
+        <v>151</v>
+      </c>
+      <c r="D32" s="282" t="s">
+        <v>1063</v>
+      </c>
+      <c r="E32" s="282" t="s">
+        <v>1260</v>
+      </c>
+      <c r="F32" s="282" t="s">
+        <v>1064</v>
+      </c>
+      <c r="G32" s="282" t="s">
+        <v>1020</v>
+      </c>
+      <c r="H32" s="282" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="21"/>
+      <c r="B33" s="294" t="s">
+        <v>1066</v>
+      </c>
+      <c r="C33" s="294"/>
+      <c r="D33" s="294"/>
+      <c r="E33" s="294"/>
+      <c r="F33" s="294"/>
+      <c r="G33" s="294"/>
+      <c r="H33" s="294"/>
+    </row>
+    <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="283" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="B34" s="295" t="s">
+        <v>952</v>
+      </c>
+      <c r="C34" s="285" t="s">
+        <v>953</v>
+      </c>
+      <c r="D34" s="306" t="n">
+        <f aca="false">E34*$C$31/8</f>
+        <v>1.0</v>
+      </c>
+      <c r="E34" s="306" t="n">
+        <f aca="false">$D$24</f>
+        <v>0.05</v>
+      </c>
+      <c r="F34" s="290" t="n">
+        <f aca="false">'ACU TAPA REGISTRO'!F69</f>
+        <v>30.42</v>
+      </c>
+      <c r="G34" s="290" t="n">
+        <f aca="false">E34*F34</f>
+        <v>1.521</v>
+      </c>
+      <c r="H34" s="149" t="s">
+        <v>1261</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="283" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="B35" s="295" t="s">
+        <v>955</v>
+      </c>
+      <c r="C35" s="285" t="s">
+        <v>953</v>
+      </c>
+      <c r="D35" s="306" t="n">
+        <f aca="false">E35*$C$31/8</f>
+        <v>2.0</v>
+      </c>
+      <c r="E35" s="306" t="n">
+        <f aca="false">$D$23</f>
+        <v>0.1</v>
+      </c>
+      <c r="F35" s="290" t="n">
+        <f aca="false">'ACU TAPA REGISTRO'!F71</f>
+        <v>20.79</v>
+      </c>
+      <c r="G35" s="290" t="n">
+        <f aca="false">E35*F35</f>
+        <v>2.079</v>
+      </c>
+      <c r="H35" s="149" t="s">
+        <v>1261</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="21"/>
+      <c r="B36" s="294" t="s">
+        <v>1068</v>
+      </c>
+      <c r="C36" s="295"/>
+      <c r="D36" s="295"/>
+      <c r="E36" s="295"/>
+      <c r="F36" s="295"/>
+      <c r="G36" s="296" t="n">
+        <f aca="false">SUM(G34:G35)</f>
+        <v>3.6</v>
+      </c>
+      <c r="H36" s="295"/>
+    </row>
+    <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="21"/>
+      <c r="B37" s="294" t="s">
+        <v>1069</v>
+      </c>
+      <c r="C37" s="294"/>
+      <c r="D37" s="294"/>
+      <c r="E37" s="294"/>
+      <c r="F37" s="294"/>
+      <c r="G37" s="294"/>
+      <c r="H37" s="294"/>
+    </row>
+    <row r="38" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="283" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="B38" s="295" t="s">
+        <v>1262</v>
+      </c>
+      <c r="C38" s="285" t="s">
+        <v>1263</v>
+      </c>
+      <c r="D38" s="295"/>
+      <c r="E38" s="306" t="n">
+        <f aca="false">$D$19</f>
+        <v>0.117752956652874</v>
+      </c>
+      <c r="F38" s="290" t="n">
+        <f aca="false">13.9/1.18</f>
+        <v>11.7796610169492</v>
+      </c>
+      <c r="G38" s="290" t="n">
+        <f aca="false">E38*F38</f>
+        <v>1.38708991311436</v>
+      </c>
+      <c r="H38" s="149" t="s">
+        <v>1264</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="283" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="B39" s="295" t="s">
+        <v>1265</v>
+      </c>
+      <c r="C39" s="285" t="s">
+        <v>981</v>
+      </c>
+      <c r="D39" s="295"/>
+      <c r="E39" s="306" t="n">
+        <f aca="false">$D$20*$D$21</f>
+        <v>0.064516</v>
+      </c>
+      <c r="F39" s="290" t="n">
+        <f aca="false">17.7/1.18</f>
+        <v>15.0</v>
+      </c>
+      <c r="G39" s="290" t="n">
+        <f aca="false">E39*F39</f>
+        <v>0.96774</v>
+      </c>
+      <c r="H39" s="149" t="s">
+        <v>1266</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="283" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="B40" s="295" t="s">
+        <v>946</v>
+      </c>
+      <c r="C40" s="285" t="s">
+        <v>167</v>
+      </c>
+      <c r="D40" s="295"/>
+      <c r="E40" s="306" t="n">
+        <f aca="false">$D$20*$D$22</f>
+        <v>0.001354836</v>
+      </c>
+      <c r="F40" s="290" t="n">
+        <f aca="false">'ACU TAPA REGISTRO'!F77</f>
+        <v>40.68</v>
+      </c>
+      <c r="G40" s="290" t="n">
+        <f aca="false">E40*F40</f>
+        <v>0.05511472848</v>
+      </c>
+      <c r="H40" s="149" t="s">
+        <v>1267</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="21"/>
+      <c r="B41" s="294" t="s">
+        <v>1071</v>
+      </c>
+      <c r="C41" s="295"/>
+      <c r="D41" s="295"/>
+      <c r="E41" s="295"/>
+      <c r="F41" s="295"/>
+      <c r="G41" s="296" t="n">
+        <f aca="false">SUM(G38:G40)</f>
+        <v>2.40994464159436</v>
+      </c>
+      <c r="H41" s="295"/>
+    </row>
+    <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="21"/>
+      <c r="B42" s="294" t="s">
+        <v>1072</v>
+      </c>
+      <c r="C42" s="294"/>
+      <c r="D42" s="294"/>
+      <c r="E42" s="294"/>
+      <c r="F42" s="294"/>
+      <c r="G42" s="294"/>
+      <c r="H42" s="294"/>
+    </row>
+    <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="283" t="n">
+        <v>6.0</v>
+      </c>
+      <c r="B43" s="295" t="s">
+        <v>969</v>
+      </c>
+      <c r="C43" s="285" t="s">
+        <v>970</v>
+      </c>
+      <c r="D43" s="295"/>
+      <c r="E43" s="284" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F43" s="290" t="n">
+        <f aca="false">+G36</f>
+        <v>3.6</v>
+      </c>
+      <c r="G43" s="290" t="n">
+        <f aca="false">E43*F43</f>
+        <v>0.108</v>
+      </c>
+      <c r="H43" s="149" t="s">
+        <v>1268</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="21"/>
+      <c r="B44" s="294" t="s">
+        <v>1075</v>
+      </c>
+      <c r="C44" s="295"/>
+      <c r="D44" s="295"/>
+      <c r="E44" s="295"/>
+      <c r="F44" s="295"/>
+      <c r="G44" s="296" t="n">
+        <f aca="false">SUM(G43:G43)</f>
+        <v>0.108</v>
+      </c>
+      <c r="H44" s="295"/>
+    </row>
+    <row r="45" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="294" t="s">
+        <v>1119</v>
+      </c>
+      <c r="B45" s="294"/>
+      <c r="C45" s="294"/>
+      <c r="D45" s="294"/>
+      <c r="E45" s="294"/>
+      <c r="F45" s="294"/>
+      <c r="G45" s="296" t="n">
+        <f aca="false">+G36+G41+G44</f>
+        <v>6.11794464159436</v>
+      </c>
+      <c r="H45" s="295"/>
+    </row>
+    <row r="46" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="294" t="s">
+        <v>1269</v>
+      </c>
+      <c r="B46" s="294"/>
+      <c r="C46" s="294"/>
+      <c r="D46" s="294"/>
+      <c r="E46" s="294"/>
+      <c r="F46" s="294"/>
+      <c r="G46" s="296" t="n">
+        <f aca="false">G45*C30</f>
+        <v>1290.75784253894</v>
+      </c>
+      <c r="H46" s="295"/>
+    </row>
+  </sheetData>
+  <mergeCells count="27">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:H2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:H3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:H4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:H5"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="C27:H27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="C28:H28"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="C29:H29"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="C30:H30"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="C31:H31"/>
+    <mergeCell ref="B33:H33"/>
+    <mergeCell ref="B37:H37"/>
+    <mergeCell ref="B42:H42"/>
+    <mergeCell ref="A45:F45"/>
+    <mergeCell ref="A46:F46"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Hogar de Refugio: hoja DESAGREGADO LLORADEROS en la planilla
Ubicacion y numero de lloraderos enlazados a METRADO LLORADEROS (157 und en 226.21 m de muro
junto a area verde, @1.50 m), componentes por lloradero de las laminas DL-01 y DL-02 (tubo PVC 3",
perforaciones, excavacion, grava, geotextil y mortero) con su total, y control con el RESUMEN.
Metrados sin cambio.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/METRADO_DRENAJE_MUJERES_VIOLENTADAS.xlsx
+++ b/entregables/METRADO_DRENAJE_MUJERES_VIOLENTADAS.xlsx
@@ -36,6 +36,7 @@
     <sheet name="DESAGREGADO TAPA REGISTRO" sheetId="26" state="visible" r:id="rId28"/>
     <sheet name="ACU JUNTA DILATACION" sheetId="27" state="visible" r:id="rId30"/>
     <sheet name="ACU JUNTA CERCO" sheetId="28" state="visible" r:id="rId31"/>
+    <sheet name="DESAGREGADO LLORADEROS" sheetId="29" state="visible" r:id="rId32"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="24" name="_xlnm.Print_Area" vbProcedure="false">'ACU CANALETAS'!$A$1:$H$111</definedName>
@@ -512,7 +513,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3401" uniqueCount="1294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3401" uniqueCount="1334">
   <si>
     <t xml:space="preserve">RESUMEN METRADOS DE DRENAJE PLUVIAL</t>
   </si>
@@ -4406,6 +4407,126 @@
   </si>
   <si>
     <t xml:space="preserve">Rendimiento (m/dia, operario de sellado)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DESAGREGADO DE LA PARTIDA 01.04.03.04.03.04 - LLORADERO DE TUBERIA PVC Ø3" C/FILTRO DE GRAVA Y GEOTEXTIL @1.50 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La partida se mide por unidad de lloradero. A: ubicacion y numero, de la hoja METRADO LLORADEROS (muros de cuneta colindantes con area verde, medidos en la planta general de drenaje; un lloradero cada 1.50 m). B: componentes de un lloradero segun las laminas DL-01 y DL-02 (tubo PVC-U Ø 3" de 0.30 m con 8 perforaciones Ø 3/8", filtro de grava de 0.30 x 0.30 x 0.30 m forrado con geotextil no tejido) por el numero de lloraderos. Celda amarilla = dato; verde = formula.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A. UBICACION Y NUMERO DE LLORADEROS (hoja METRADO LLORADEROS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EJE Y TRAMO (progresivas de la cuneta)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LONGITUD JUNTO A AREA VERDE (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESPACIAM. (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">planta general de drenaje; N° = REDONDEAR.MAS(L / 1.50)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL (und de la partida)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B. DATOS DEL DETALLE (laminas DL-01 y DL-02)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lado del filtro localizado (cubo de grava forrado con geotextil)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DL-02 A: filtro 0.30 x 0.30 x 0.30 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Longitud del tubo PVC-U Ø 3" por lloradero</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DL-02 B: 0.10 en el muro + 0.20 perforado dentro del filtro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perforaciones Ø 3/8" por fila</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DL-02 B: 4 perforaciones @0.05 por fila</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filas de perforaciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DL-02 B: 2 filas a 120 grados, simetricas respecto al fondo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desperdicio de grava (acomodo y perdidas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">criterio de obra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traslapes del geotextil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DL-01 etapa 3: traslape de 0.10 m al cerrar el filtro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mortero 1:3 de sellado alrededor del tubo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">anillo de 0.02 m en las dos caras del muro (DL-02)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C. COMPONENTES DE UN LLORADERO Y TOTAL DE LA PARTIDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POR LLORADERO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N° LLORADEROS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tubo PVC-U Ø 3" para desague (NTP 399.003)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DL-02 B; sale de tubos de 3 m (10 lloraderos por tubo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perforaciones Ø 3/8" en el tramo dentro del filtro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DL-02 B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excavacion local del hueco del filtro (lado^3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DL-01 etapa 1; incluida en la mano de obra del ACU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grava filtrante (ripio) 20 a 40 mm: lado^3 + desperdicio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DL-01 etapa 2; DL-02 A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Geotextil no tejido clase 2: 6 caras del cubo + traslapes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DL-01 etapa 3; DL-02 A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DL-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D. CONTROL CON EL RESUMEN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RESUMEN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01.04.03.04.03.04 LLORADERO DE TUBERIA PVC Ø3" C/FILTRO DE GRAVA Y GEOTEXTIL @1.50 m</t>
   </si>
 </sst>
 </file>
@@ -34082,6 +34203,959 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:H46"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="44"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="277" t="s">
+        <v>1294</v>
+      </c>
+      <c r="B1" s="277"/>
+      <c r="C1" s="277"/>
+      <c r="D1" s="277"/>
+      <c r="E1" s="277"/>
+      <c r="F1" s="277"/>
+      <c r="G1" s="277"/>
+      <c r="H1" s="277"/>
+    </row>
+    <row r="2" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="278" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="278"/>
+      <c r="C2" s="279" t="str">
+        <f aca="false">+RESUMEN!B4</f>
+        <v>GERENCIA TERRITORIAL BAJO MAYO - TARAPOTO</v>
+      </c>
+      <c r="D2" s="279"/>
+      <c r="E2" s="279"/>
+      <c r="F2" s="279"/>
+      <c r="G2" s="279"/>
+      <c r="H2" s="279"/>
+    </row>
+    <row r="3" customFormat="false" ht="58.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="278" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="278"/>
+      <c r="C3" s="279" t="str">
+        <f aca="false">+RESUMEN!B5</f>
+        <v>“CREACIÓN DEL SERVICIO DE PROTECCIÓN A MUJERES VÍCTIMAS DE VIOLENCIA EN SITUACIÓN DE RIESGO DE FEMINICIDIO O PELIGRE SU INTEGRIDAD Y/O SALUD FÍSICA Y/O MENTAL EN HOGAR DE REFUGIO TEMPORAL DISTRITO DE MORALES DE LA PROVINCIA DE SAN MARTÍN DEL DEPARTAMENTO DE SAN MARTÍN”, con CUI N.° 2675514</v>
+      </c>
+      <c r="D3" s="279"/>
+      <c r="E3" s="279"/>
+      <c r="F3" s="279"/>
+      <c r="G3" s="279"/>
+      <c r="H3" s="279"/>
+    </row>
+    <row r="4" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="278" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="278"/>
+      <c r="C4" s="279" t="str">
+        <f aca="false">+RESUMEN!B6</f>
+        <v>SAN MARTIN - SAN MARTIN - MORALES</v>
+      </c>
+      <c r="D4" s="279"/>
+      <c r="E4" s="279"/>
+      <c r="F4" s="279"/>
+      <c r="G4" s="279"/>
+      <c r="H4" s="279"/>
+    </row>
+    <row r="5" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="278" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="278"/>
+      <c r="C5" s="280" t="n">
+        <f aca="false">+RESUMEN!B7</f>
+        <v>46266</v>
+      </c>
+      <c r="D5" s="280"/>
+      <c r="E5" s="280"/>
+      <c r="F5" s="280"/>
+      <c r="G5" s="280"/>
+      <c r="H5" s="280"/>
+    </row>
+    <row r="7" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="281" t="s">
+        <v>1295</v>
+      </c>
+      <c r="B7" s="281"/>
+      <c r="C7" s="281"/>
+      <c r="D7" s="281"/>
+      <c r="E7" s="281"/>
+      <c r="F7" s="281"/>
+      <c r="G7" s="281"/>
+      <c r="H7" s="281"/>
+    </row>
+    <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="294" t="s">
+        <v>1296</v>
+      </c>
+      <c r="B9" s="294"/>
+      <c r="C9" s="294"/>
+      <c r="D9" s="294"/>
+      <c r="E9" s="294"/>
+      <c r="F9" s="294"/>
+      <c r="G9" s="294"/>
+      <c r="H9" s="294"/>
+    </row>
+    <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="282" t="s">
+        <v>331</v>
+      </c>
+      <c r="B10" s="282" t="s">
+        <v>1297</v>
+      </c>
+      <c r="C10" s="282" t="s">
+        <v>460</v>
+      </c>
+      <c r="D10" s="282" t="s">
+        <v>1298</v>
+      </c>
+      <c r="E10" s="282" t="s">
+        <v>1299</v>
+      </c>
+      <c r="F10" s="282" t="s">
+        <v>463</v>
+      </c>
+      <c r="G10" s="282"/>
+      <c r="H10" s="282" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="283" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="B11" s="149" t="str">
+        <f aca="false">'METRADO LLORADEROS'!B7&amp;": "&amp;'METRADO LLORADEROS'!C7</f>
+        <v>EJE 01: 0+000.00 a 0+037.00</v>
+      </c>
+      <c r="C11" s="285" t="str">
+        <f aca="false">'METRADO LLORADEROS'!D7</f>
+        <v>LADO ESTE</v>
+      </c>
+      <c r="D11" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!E7</f>
+        <v>37.0</v>
+      </c>
+      <c r="E11" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!F7</f>
+        <v>1.5</v>
+      </c>
+      <c r="F11" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!G7</f>
+        <v>25.0</v>
+      </c>
+      <c r="G11" s="295"/>
+      <c r="H11" s="149" t="s">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="283" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="B12" s="149" t="str">
+        <f aca="false">'METRADO LLORADEROS'!B8&amp;": "&amp;'METRADO LLORADEROS'!C8</f>
+        <v>EJE 01: 0+032.25 a 0+037.00</v>
+      </c>
+      <c r="C12" s="285" t="str">
+        <f aca="false">'METRADO LLORADEROS'!D8</f>
+        <v>LADO OESTE</v>
+      </c>
+      <c r="D12" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!E8</f>
+        <v>4.75</v>
+      </c>
+      <c r="E12" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!F8</f>
+        <v>1.5</v>
+      </c>
+      <c r="F12" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!G8</f>
+        <v>4.0</v>
+      </c>
+      <c r="G12" s="295"/>
+      <c r="H12" s="149" t="s">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="283" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="B13" s="149" t="str">
+        <f aca="false">'METRADO LLORADEROS'!B9&amp;": "&amp;'METRADO LLORADEROS'!C9</f>
+        <v>EJE 02: 0+040.62 a 0+045.37</v>
+      </c>
+      <c r="C13" s="285" t="str">
+        <f aca="false">'METRADO LLORADEROS'!D9</f>
+        <v>LADO SUR</v>
+      </c>
+      <c r="D13" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!E9</f>
+        <v>4.75</v>
+      </c>
+      <c r="E13" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!F9</f>
+        <v>1.5</v>
+      </c>
+      <c r="F13" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!G9</f>
+        <v>4.0</v>
+      </c>
+      <c r="G13" s="295"/>
+      <c r="H13" s="149" t="s">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="283" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="B14" s="149" t="str">
+        <f aca="false">'METRADO LLORADEROS'!B10&amp;": "&amp;'METRADO LLORADEROS'!C10</f>
+        <v>EJE 07: 0+040.62 a 0+042.87</v>
+      </c>
+      <c r="C14" s="285" t="str">
+        <f aca="false">'METRADO LLORADEROS'!D10</f>
+        <v>LADO SUR</v>
+      </c>
+      <c r="D14" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!E10</f>
+        <v>2.25</v>
+      </c>
+      <c r="E14" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!F10</f>
+        <v>1.5</v>
+      </c>
+      <c r="F14" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!G10</f>
+        <v>2.0</v>
+      </c>
+      <c r="G14" s="295"/>
+      <c r="H14" s="149" t="s">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="283" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="B15" s="149" t="str">
+        <f aca="false">'METRADO LLORADEROS'!B11&amp;": "&amp;'METRADO LLORADEROS'!C11</f>
+        <v>EJE 07: 0+123.97 a 0+125.70</v>
+      </c>
+      <c r="C15" s="285" t="str">
+        <f aca="false">'METRADO LLORADEROS'!D11</f>
+        <v>LADO ESTE</v>
+      </c>
+      <c r="D15" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!E11</f>
+        <v>1.73</v>
+      </c>
+      <c r="E15" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!F11</f>
+        <v>1.5</v>
+      </c>
+      <c r="F15" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!G11</f>
+        <v>2.0</v>
+      </c>
+      <c r="G15" s="295"/>
+      <c r="H15" s="149" t="s">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="283" t="n">
+        <v>6.0</v>
+      </c>
+      <c r="B16" s="149" t="str">
+        <f aca="false">'METRADO LLORADEROS'!B12&amp;": "&amp;'METRADO LLORADEROS'!C12</f>
+        <v>EJE 07: 0+123.97 a 0+125.70</v>
+      </c>
+      <c r="C16" s="285" t="str">
+        <f aca="false">'METRADO LLORADEROS'!D12</f>
+        <v>LADO OESTE</v>
+      </c>
+      <c r="D16" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!E12</f>
+        <v>1.73</v>
+      </c>
+      <c r="E16" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!F12</f>
+        <v>1.5</v>
+      </c>
+      <c r="F16" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!G12</f>
+        <v>2.0</v>
+      </c>
+      <c r="G16" s="295"/>
+      <c r="H16" s="149" t="s">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="283" t="n">
+        <v>7.0</v>
+      </c>
+      <c r="B17" s="149" t="str">
+        <f aca="false">'METRADO LLORADEROS'!B13&amp;": "&amp;'METRADO LLORADEROS'!C13</f>
+        <v>EJE 09: 0+000.50 a 0+005.00</v>
+      </c>
+      <c r="C17" s="285" t="str">
+        <f aca="false">'METRADO LLORADEROS'!D13</f>
+        <v>LADO SUR</v>
+      </c>
+      <c r="D17" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!E13</f>
+        <v>4.5</v>
+      </c>
+      <c r="E17" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!F13</f>
+        <v>1.5</v>
+      </c>
+      <c r="F17" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!G13</f>
+        <v>3.0</v>
+      </c>
+      <c r="G17" s="295"/>
+      <c r="H17" s="149" t="s">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="283" t="n">
+        <v>8.0</v>
+      </c>
+      <c r="B18" s="149" t="str">
+        <f aca="false">'METRADO LLORADEROS'!B14&amp;": "&amp;'METRADO LLORADEROS'!C14</f>
+        <v>EJE 11: 0+069.05 a 0+071.30</v>
+      </c>
+      <c r="C18" s="285" t="str">
+        <f aca="false">'METRADO LLORADEROS'!D14</f>
+        <v>LADO ESTE</v>
+      </c>
+      <c r="D18" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!E14</f>
+        <v>2.25</v>
+      </c>
+      <c r="E18" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!F14</f>
+        <v>1.5</v>
+      </c>
+      <c r="F18" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!G14</f>
+        <v>2.0</v>
+      </c>
+      <c r="G18" s="295"/>
+      <c r="H18" s="149" t="s">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="283" t="n">
+        <v>9.0</v>
+      </c>
+      <c r="B19" s="149" t="str">
+        <f aca="false">'METRADO LLORADEROS'!B15&amp;": "&amp;'METRADO LLORADEROS'!C15</f>
+        <v>EJE 11: 0+039.50 a 0+062.75</v>
+      </c>
+      <c r="C19" s="285" t="str">
+        <f aca="false">'METRADO LLORADEROS'!D15</f>
+        <v>LADO OESTE</v>
+      </c>
+      <c r="D19" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!E15</f>
+        <v>23.25</v>
+      </c>
+      <c r="E19" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!F15</f>
+        <v>1.5</v>
+      </c>
+      <c r="F19" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!G15</f>
+        <v>16.0</v>
+      </c>
+      <c r="G19" s="295"/>
+      <c r="H19" s="149" t="s">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="283" t="n">
+        <v>10.0</v>
+      </c>
+      <c r="B20" s="149" t="str">
+        <f aca="false">'METRADO LLORADEROS'!B16&amp;": "&amp;'METRADO LLORADEROS'!C16</f>
+        <v>EJE 11: 0+066.80 a 0+071.30</v>
+      </c>
+      <c r="C20" s="285" t="str">
+        <f aca="false">'METRADO LLORADEROS'!D16</f>
+        <v>LADO OESTE</v>
+      </c>
+      <c r="D20" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!E16</f>
+        <v>4.5</v>
+      </c>
+      <c r="E20" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!F16</f>
+        <v>1.5</v>
+      </c>
+      <c r="F20" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!G16</f>
+        <v>3.0</v>
+      </c>
+      <c r="G20" s="295"/>
+      <c r="H20" s="149" t="s">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="283" t="n">
+        <v>11.0</v>
+      </c>
+      <c r="B21" s="149" t="str">
+        <f aca="false">'METRADO LLORADEROS'!B17&amp;": "&amp;'METRADO LLORADEROS'!C17</f>
+        <v>EJE 12: 0+078.50 a 0+109.00</v>
+      </c>
+      <c r="C21" s="285" t="str">
+        <f aca="false">'METRADO LLORADEROS'!D17</f>
+        <v>LADO ESTE</v>
+      </c>
+      <c r="D21" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!E17</f>
+        <v>30.5</v>
+      </c>
+      <c r="E21" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!F17</f>
+        <v>1.5</v>
+      </c>
+      <c r="F21" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!G17</f>
+        <v>21.0</v>
+      </c>
+      <c r="G21" s="295"/>
+      <c r="H21" s="149" t="s">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="283" t="n">
+        <v>12.0</v>
+      </c>
+      <c r="B22" s="149" t="str">
+        <f aca="false">'METRADO LLORADEROS'!B18&amp;": "&amp;'METRADO LLORADEROS'!C18</f>
+        <v>EJE 12: 0+000.00 a 0+109.00</v>
+      </c>
+      <c r="C22" s="285" t="str">
+        <f aca="false">'METRADO LLORADEROS'!D18</f>
+        <v>LADO OESTE</v>
+      </c>
+      <c r="D22" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!E18</f>
+        <v>109.0</v>
+      </c>
+      <c r="E22" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!F18</f>
+        <v>1.5</v>
+      </c>
+      <c r="F22" s="290" t="n">
+        <f aca="false">'METRADO LLORADEROS'!G18</f>
+        <v>73.0</v>
+      </c>
+      <c r="G22" s="295"/>
+      <c r="H22" s="149" t="s">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="21"/>
+      <c r="B23" s="294" t="s">
+        <v>1301</v>
+      </c>
+      <c r="C23" s="295"/>
+      <c r="D23" s="296" t="n">
+        <f aca="false">SUM(D11:D22)</f>
+        <v>226.21</v>
+      </c>
+      <c r="E23" s="295"/>
+      <c r="F23" s="296" t="n">
+        <f aca="false">SUM(F11:F22)</f>
+        <v>157.0</v>
+      </c>
+      <c r="G23" s="295"/>
+      <c r="H23" s="295"/>
+    </row>
+    <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="294" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B25" s="294"/>
+      <c r="C25" s="294"/>
+      <c r="D25" s="294"/>
+      <c r="E25" s="294"/>
+      <c r="F25" s="294"/>
+      <c r="G25" s="294"/>
+      <c r="H25" s="294"/>
+    </row>
+    <row r="26" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="282" t="s">
+        <v>331</v>
+      </c>
+      <c r="B26" s="282" t="s">
+        <v>1082</v>
+      </c>
+      <c r="C26" s="282" t="s">
+        <v>151</v>
+      </c>
+      <c r="D26" s="282" t="s">
+        <v>292</v>
+      </c>
+      <c r="E26" s="282"/>
+      <c r="F26" s="282"/>
+      <c r="G26" s="282"/>
+      <c r="H26" s="282" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="283" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="B27" s="149" t="s">
+        <v>1303</v>
+      </c>
+      <c r="C27" s="285" t="s">
+        <v>57</v>
+      </c>
+      <c r="D27" s="307" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E27" s="295"/>
+      <c r="F27" s="295"/>
+      <c r="G27" s="295"/>
+      <c r="H27" s="149" t="s">
+        <v>1304</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="283" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="B28" s="149" t="s">
+        <v>1305</v>
+      </c>
+      <c r="C28" s="285" t="s">
+        <v>57</v>
+      </c>
+      <c r="D28" s="307" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E28" s="295"/>
+      <c r="F28" s="295"/>
+      <c r="G28" s="295"/>
+      <c r="H28" s="149" t="s">
+        <v>1306</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="283" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="B29" s="149" t="s">
+        <v>1307</v>
+      </c>
+      <c r="C29" s="285" t="s">
+        <v>60</v>
+      </c>
+      <c r="D29" s="307" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="E29" s="295"/>
+      <c r="F29" s="295"/>
+      <c r="G29" s="295"/>
+      <c r="H29" s="149" t="s">
+        <v>1308</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="283" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="B30" s="149" t="s">
+        <v>1309</v>
+      </c>
+      <c r="C30" s="285" t="s">
+        <v>60</v>
+      </c>
+      <c r="D30" s="307" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="E30" s="295"/>
+      <c r="F30" s="295"/>
+      <c r="G30" s="295"/>
+      <c r="H30" s="149" t="s">
+        <v>1310</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="283" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="B31" s="149" t="s">
+        <v>1311</v>
+      </c>
+      <c r="C31" s="285" t="s">
+        <v>523</v>
+      </c>
+      <c r="D31" s="307" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E31" s="295"/>
+      <c r="F31" s="295"/>
+      <c r="G31" s="295"/>
+      <c r="H31" s="149" t="s">
+        <v>1312</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="283" t="n">
+        <v>6.0</v>
+      </c>
+      <c r="B32" s="149" t="s">
+        <v>1313</v>
+      </c>
+      <c r="C32" s="285" t="s">
+        <v>523</v>
+      </c>
+      <c r="D32" s="307" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E32" s="295"/>
+      <c r="F32" s="295"/>
+      <c r="G32" s="295"/>
+      <c r="H32" s="149" t="s">
+        <v>1314</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="283" t="n">
+        <v>7.0</v>
+      </c>
+      <c r="B33" s="149" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C33" s="285" t="s">
+        <v>167</v>
+      </c>
+      <c r="D33" s="307" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="E33" s="295"/>
+      <c r="F33" s="295"/>
+      <c r="G33" s="295"/>
+      <c r="H33" s="149" t="s">
+        <v>1316</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="294" t="s">
+        <v>1317</v>
+      </c>
+      <c r="B35" s="294"/>
+      <c r="C35" s="294"/>
+      <c r="D35" s="294"/>
+      <c r="E35" s="294"/>
+      <c r="F35" s="294"/>
+      <c r="G35" s="294"/>
+      <c r="H35" s="294"/>
+    </row>
+    <row r="36" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="282" t="s">
+        <v>331</v>
+      </c>
+      <c r="B36" s="282" t="s">
+        <v>992</v>
+      </c>
+      <c r="C36" s="282" t="s">
+        <v>151</v>
+      </c>
+      <c r="D36" s="282" t="s">
+        <v>1318</v>
+      </c>
+      <c r="E36" s="282" t="s">
+        <v>1319</v>
+      </c>
+      <c r="F36" s="282" t="s">
+        <v>150</v>
+      </c>
+      <c r="G36" s="282"/>
+      <c r="H36" s="282" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="283" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="B37" s="149" t="s">
+        <v>1320</v>
+      </c>
+      <c r="C37" s="285" t="s">
+        <v>57</v>
+      </c>
+      <c r="D37" s="306" t="n">
+        <f aca="false">$D$28</f>
+        <v>0.3</v>
+      </c>
+      <c r="E37" s="290" t="n">
+        <f aca="false">+$F$23</f>
+        <v>157.0</v>
+      </c>
+      <c r="F37" s="306" t="n">
+        <f aca="false">D37*E37</f>
+        <v>47.1</v>
+      </c>
+      <c r="G37" s="295"/>
+      <c r="H37" s="149" t="s">
+        <v>1321</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="283" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="B38" s="149" t="s">
+        <v>1322</v>
+      </c>
+      <c r="C38" s="285" t="s">
+        <v>60</v>
+      </c>
+      <c r="D38" s="306" t="n">
+        <f aca="false">$D$29*$D$30</f>
+        <v>8.0</v>
+      </c>
+      <c r="E38" s="290" t="n">
+        <f aca="false">+$F$23</f>
+        <v>157.0</v>
+      </c>
+      <c r="F38" s="306" t="n">
+        <f aca="false">D38*E38</f>
+        <v>1256.0</v>
+      </c>
+      <c r="G38" s="295"/>
+      <c r="H38" s="149" t="s">
+        <v>1323</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="283" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="B39" s="149" t="s">
+        <v>1324</v>
+      </c>
+      <c r="C39" s="285" t="s">
+        <v>167</v>
+      </c>
+      <c r="D39" s="306" t="n">
+        <f aca="false">$D$27^3</f>
+        <v>0.027</v>
+      </c>
+      <c r="E39" s="290" t="n">
+        <f aca="false">+$F$23</f>
+        <v>157.0</v>
+      </c>
+      <c r="F39" s="306" t="n">
+        <f aca="false">D39*E39</f>
+        <v>4.239</v>
+      </c>
+      <c r="G39" s="295"/>
+      <c r="H39" s="149" t="s">
+        <v>1325</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="283" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="B40" s="149" t="s">
+        <v>1326</v>
+      </c>
+      <c r="C40" s="285" t="s">
+        <v>167</v>
+      </c>
+      <c r="D40" s="306" t="n">
+        <f aca="false">$D$27^3*(1+$D$31)</f>
+        <v>0.0297</v>
+      </c>
+      <c r="E40" s="290" t="n">
+        <f aca="false">+$F$23</f>
+        <v>157.0</v>
+      </c>
+      <c r="F40" s="306" t="n">
+        <f aca="false">D40*E40</f>
+        <v>4.6629</v>
+      </c>
+      <c r="G40" s="295"/>
+      <c r="H40" s="149" t="s">
+        <v>1327</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="283" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="B41" s="149" t="s">
+        <v>1328</v>
+      </c>
+      <c r="C41" s="285" t="s">
+        <v>168</v>
+      </c>
+      <c r="D41" s="306" t="n">
+        <f aca="false">6*$D$27^2*(1+$D$32)</f>
+        <v>0.594</v>
+      </c>
+      <c r="E41" s="290" t="n">
+        <f aca="false">+$F$23</f>
+        <v>157.0</v>
+      </c>
+      <c r="F41" s="306" t="n">
+        <f aca="false">D41*E41</f>
+        <v>93.258</v>
+      </c>
+      <c r="G41" s="295"/>
+      <c r="H41" s="149" t="s">
+        <v>1329</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="283" t="n">
+        <v>6.0</v>
+      </c>
+      <c r="B42" s="149" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C42" s="285" t="s">
+        <v>167</v>
+      </c>
+      <c r="D42" s="306" t="n">
+        <f aca="false">$D$33</f>
+        <v>0.0005</v>
+      </c>
+      <c r="E42" s="290" t="n">
+        <f aca="false">+$F$23</f>
+        <v>157.0</v>
+      </c>
+      <c r="F42" s="306" t="n">
+        <f aca="false">D42*E42</f>
+        <v>0.0785</v>
+      </c>
+      <c r="G42" s="295"/>
+      <c r="H42" s="149" t="s">
+        <v>1330</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="294" t="s">
+        <v>1331</v>
+      </c>
+      <c r="B44" s="294"/>
+      <c r="C44" s="294"/>
+      <c r="D44" s="294"/>
+      <c r="E44" s="294"/>
+      <c r="F44" s="294"/>
+      <c r="G44" s="294"/>
+      <c r="H44" s="294"/>
+    </row>
+    <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="282"/>
+      <c r="B45" s="282" t="s">
+        <v>891</v>
+      </c>
+      <c r="C45" s="282" t="s">
+        <v>151</v>
+      </c>
+      <c r="D45" s="282"/>
+      <c r="E45" s="282" t="s">
+        <v>1177</v>
+      </c>
+      <c r="F45" s="282" t="s">
+        <v>1332</v>
+      </c>
+      <c r="G45" s="282" t="s">
+        <v>1179</v>
+      </c>
+      <c r="H45" s="282"/>
+    </row>
+    <row r="46" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="21"/>
+      <c r="B46" s="149" t="s">
+        <v>1333</v>
+      </c>
+      <c r="C46" s="285" t="s">
+        <v>60</v>
+      </c>
+      <c r="D46" s="295"/>
+      <c r="E46" s="306" t="n">
+        <f aca="false">+$F$23</f>
+        <v>157.0</v>
+      </c>
+      <c r="F46" s="306" t="n">
+        <f aca="false">+RESUMEN!D32</f>
+        <v>157.0</v>
+      </c>
+      <c r="G46" s="283" t="str">
+        <f aca="false">IF(ABS(E46-F46)&lt;0.001,"CONFORME","REVISAR")</f>
+        <v>CONFORME</v>
+      </c>
+      <c r="H46" s="295"/>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:H2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:H3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:H4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:H5"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A44:H44"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">

</xml_diff>

<commit_message>
Hogar de Refugio: ventana de salida de la caja CC al R-01 del CAR Mujeres de 1.50 x 0.43
El alto de la ventana es el alto interior del colector receptor en su R-01 (losa 259.25 - 0.10 - fondo 258.72).
DP-07 la dibujaba de 0.60 y la planilla descontaba 0.842; el perfil ya la dibujaba de 0.43.
Concreto del colector y cajas: 58.31 -> 58.41 m3.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/METRADO_DRENAJE_MUJERES_VIOLENTADAS.xlsx
+++ b/entregables/METRADO_DRENAJE_MUJERES_VIOLENTADAS.xlsx
@@ -515,7 +515,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3401" uniqueCount="1480">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3401" uniqueCount="1481">
   <si>
     <t xml:space="preserve">RESUMEN METRADOS DE DRENAJE PLUVIAL</t>
   </si>
@@ -4969,6 +4969,9 @@
   </si>
   <si>
     <t xml:space="preserve">DD-03 C; EG-2013 MTC, Seccion 510</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caja de caida CC: descuento ventana de salida (alto = interior del R-01 del CAR Mujeres: losa 259.25 - 0.10 - fondo)</t>
   </si>
 </sst>
 </file>
@@ -8256,7 +8259,7 @@
       </c>
       <c r="D66" s="16" t="n">
         <f aca="false">+'PLANILLA GENERAL DE METRADOS'!K240</f>
-        <v>58.3136159999999</v>
+        <v>58.4063159999999</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15045,7 +15048,7 @@
     <row r="38" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="21"/>
       <c r="B38" s="149" t="s">
-        <v>757</v>
+        <v>1480</v>
       </c>
       <c r="C38" s="283" t="s">
         <v>729</v>
@@ -15059,8 +15062,8 @@
         <v>0.15</v>
       </c>
       <c r="F38" s="287" t="n">
-        <f aca="false">'COLECTOR PARAMETROS'!$C$57+0.5-'COLECTOR PARAMETROS'!$C$56</f>
-        <v>0.841999999999985</v>
+        <f aca="false">259.25-0.1-'COLECTOR PARAMETROS'!$C$56</f>
+        <v>0.42999999999995</v>
       </c>
       <c r="G38" s="298" t="n">
         <v>-1</v>
@@ -15069,7 +15072,7 @@
       <c r="I38" s="21"/>
       <c r="J38" s="290" t="n">
         <f aca="false">D38*E38*F38*G38</f>
-        <v>-0.189449999999997</v>
+        <v>-0.0967499999999887</v>
       </c>
       <c r="K38" s="21"/>
       <c r="L38" s="21"/>
@@ -15367,7 +15370,7 @@
       </c>
       <c r="J47" s="293" t="n">
         <f aca="false">SUM(J21:J46)</f>
-        <v>4.53719999999988</v>
+        <v>4.62989999999989</v>
       </c>
       <c r="K47" s="293" t="n">
         <f aca="false">SUM(K21:K46)</f>
@@ -15472,11 +15475,11 @@
       </c>
       <c r="H52" s="290" t="n">
         <f aca="false">J47</f>
-        <v>4.53719999999988</v>
+        <v>4.62989999999989</v>
       </c>
       <c r="I52" s="296" t="n">
         <f aca="false">G52+H52</f>
-        <v>35.8622159999999</v>
+        <v>35.9549159999999</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -21833,7 +21836,7 @@
       <c r="J240" s="25"/>
       <c r="K240" s="25" t="n">
         <f aca="false">SUM(J241:J271)</f>
-        <v>58.3136159999999</v>
+        <v>58.4063159999999</v>
       </c>
       <c r="L240" s="24" t="s">
         <v>25</v>
@@ -22228,7 +22231,7 @@
       <c r="I259" s="27"/>
       <c r="J259" s="27" t="n">
         <f aca="false">SUM('COLECTOR CONCRETO'!J33:J43)</f>
-        <v>2.91449999999992</v>
+        <v>3.00719999999993</v>
       </c>
       <c r="K259" s="27"/>
       <c r="L259" s="26"/>
@@ -26673,7 +26676,7 @@
       </c>
       <c r="D19" s="290" t="n">
         <f aca="false">SUM('PLANILLA GENERAL DE METRADOS'!J251:J259)</f>
-        <v>35.8622159999999</v>
+        <v>35.9549159999999</v>
       </c>
       <c r="E19" s="295" t="s">
         <v>944</v>
@@ -26686,7 +26689,7 @@
       </c>
       <c r="H19" s="296" t="n">
         <f aca="false">G19*$D$19</f>
-        <v>348.939361679999</v>
+        <v>349.841332679999</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26705,7 +26708,7 @@
       </c>
       <c r="H20" s="296" t="n">
         <f aca="false">G20*$D$19</f>
-        <v>18.6483523199999</v>
+        <v>18.6965563199999</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26724,7 +26727,7 @@
       </c>
       <c r="H21" s="296" t="n">
         <f aca="false">G21*$D$19</f>
-        <v>19.0069744799999</v>
+        <v>19.0561054799999</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26743,7 +26746,7 @@
       </c>
       <c r="H22" s="296" t="n">
         <f aca="false">G22*$D$19</f>
-        <v>6.67037217599998</v>
+        <v>6.68761437599998</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26762,7 +26765,7 @@
       </c>
       <c r="H23" s="296" t="n">
         <f aca="false">G23*$D$19</f>
-        <v>35.8622159999999</v>
+        <v>35.9549159999999</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26781,7 +26784,7 @@
       </c>
       <c r="H24" s="296" t="n">
         <f aca="false">G24*$D$19</f>
-        <v>35.8622159999999</v>
+        <v>35.9549159999999</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26800,7 +26803,7 @@
       </c>
       <c r="H25" s="296" t="n">
         <f aca="false">G25*$D$19</f>
-        <v>35.8622159999999</v>
+        <v>35.9549159999999</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26819,7 +26822,7 @@
       </c>
       <c r="H26" s="296" t="n">
         <f aca="false">G26*$D$19</f>
-        <v>35.8622159999999</v>
+        <v>35.9549159999999</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26838,7 +26841,7 @@
       </c>
       <c r="H27" s="296" t="n">
         <f aca="false">G27*$D$19</f>
-        <v>286.897727999999</v>
+        <v>287.639327999999</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Tapa ciega de concreto armado en los 3 CAR: DP-06B, DD-01, DD-02, isometricos, metrado de Refugio y Varones
- Tapa ciega 0.68x0.68x0.08 vaciada aparte en obra, parrilla 3/8" @0.10 y 2 asas de fierro liso 1/2" en cajuelas, sin marco ni contramarco metalico; asiento en rebaje de concreto 0.70x0.70x0.08 de la losa (luz libre 0.60).
- DP-06B nuevo para Hogar de Refugio (CUI 2675514), CAR Varones (CUI 2705619) y CAR Mujeres (CUI 2717013), sueltos y dentro de cada juego de planos, con vistas previas.
- Metrado y ACU de la tapa actualizados solo en Refugio y Varones; el metrado de CAR Mujeres no se toca.
- DD-01, DD-02, DP-06D, DP-08, DP-09, DA-03, especificaciones y memorias coherentes con la tapa ciega.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/METRADO_DRENAJE_MUJERES_VIOLENTADAS.xlsx
+++ b/entregables/METRADO_DRENAJE_MUJERES_VIOLENTADAS.xlsx
@@ -515,7 +515,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3401" uniqueCount="1566">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3401" uniqueCount="1568">
   <si>
     <t xml:space="preserve">RESUMEN METRADOS DE DRENAJE PLUVIAL</t>
   </si>
@@ -5227,6 +5227,12 @@
   </si>
   <si>
     <t xml:space="preserve">No hay angulos, soldadura ni pintura: la tapa es ciega de concreto armado (lamina DP-06B rev. 02). El rebaje de asiento y el borde engrosado de la abertura se metran con el concreto de la losa del colector (hoja COLECTOR CONCRETO).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lamina DP-06B rev. 02: agarre 0.15 + 2 patas de 0.02 + 2 ganchos de 0.15 (0.49, se toma 0.50)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REGISTROS DE LIMPIEZA Y TAPAS - lamina DP-06B: refuerzo de borde de la abertura, parrilla de la tapa, asas de la tapa ciega (cantidad de registros de la hoja COLECTOR REGISTROS Y TAPAS)</t>
   </si>
 </sst>
 </file>
@@ -12413,7 +12419,7 @@
         <v>57</v>
       </c>
       <c r="E39" s="286" t="s">
-        <v>1488</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -25266,7 +25272,7 @@
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="294" t="s">
-        <v>839</v>
+        <v>1567</v>
       </c>
       <c r="B31" s="294"/>
       <c r="C31" s="294"/>

</xml_diff>